<commit_message>
Tracker: add Business OCR (now 3 boards × 30 lessons = 90 rows on Business Studies sheet)
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/gcse-subject-tracker.xlsx
+++ b/data/gcse-subject-tracker.xlsx
@@ -32,7 +32,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Health &amp; Social Care'!$A$1:$H$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Hospitality &amp; Catering'!$A$1:$H$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Music Technology'!$A$1:$H$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Business Studies'!$A$1:$H$61</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Business Studies'!$A$1:$H$91</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -12169,7 +12169,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H61"/>
+  <dimension ref="A1:H91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -14144,8 +14144,968 @@
       <c r="G61" s="2" t="inlineStr"/>
       <c r="H61" s="2" t="inlineStr"/>
     </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>Business Studies</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Business Activity, Marketing &amp; People</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E62" s="12" t="inlineStr">
+        <is>
+          <t>Enterprise, Entrepreneurs &amp; Risk and Reward</t>
+        </is>
+      </c>
+      <c r="F62" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr"/>
+      <c r="H62" s="2" t="inlineStr"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>Business Studies</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>Business Activity, Marketing &amp; People</t>
+        </is>
+      </c>
+      <c r="D63" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E63" s="12" t="inlineStr">
+        <is>
+          <t>Business Planning</t>
+        </is>
+      </c>
+      <c r="F63" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr"/>
+      <c r="H63" s="2" t="inlineStr"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>Business Studies</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Business Activity, Marketing &amp; People</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E64" s="12" t="inlineStr">
+        <is>
+          <t>Business Ownership &amp; Limited Liability</t>
+        </is>
+      </c>
+      <c r="F64" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr"/>
+      <c r="H64" s="2" t="inlineStr"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>Business Studies</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>Business Activity, Marketing &amp; People</t>
+        </is>
+      </c>
+      <c r="D65" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E65" s="12" t="inlineStr">
+        <is>
+          <t>Business Aims &amp; Objectives</t>
+        </is>
+      </c>
+      <c r="F65" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr"/>
+      <c r="H65" s="2" t="inlineStr"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>Business Studies</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Business Activity, Marketing &amp; People</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E66" s="12" t="inlineStr">
+        <is>
+          <t>Stakeholders in Business</t>
+        </is>
+      </c>
+      <c r="F66" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr"/>
+      <c r="H66" s="2" t="inlineStr"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>Business Studies</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>Business Activity, Marketing &amp; People</t>
+        </is>
+      </c>
+      <c r="D67" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="E67" s="12" t="inlineStr">
+        <is>
+          <t>Business Growth</t>
+        </is>
+      </c>
+      <c r="F67" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr"/>
+      <c r="H67" s="2" t="inlineStr"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>Business Studies</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>Business Activity, Marketing &amp; People</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="E68" s="12" t="inlineStr">
+        <is>
+          <t>Role &amp; Purpose of Marketing</t>
+        </is>
+      </c>
+      <c r="F68" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr"/>
+      <c r="H68" s="2" t="inlineStr"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>Business Studies</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>Business Activity, Marketing &amp; People</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E69" s="12" t="inlineStr">
+        <is>
+          <t>Market Research</t>
+        </is>
+      </c>
+      <c r="F69" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr"/>
+      <c r="H69" s="2" t="inlineStr"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>Business Studies</t>
+        </is>
+      </c>
+      <c r="B70" s="2" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+      <c r="C70" s="2" t="inlineStr">
+        <is>
+          <t>Business Activity, Marketing &amp; People</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E70" s="12" t="inlineStr">
+        <is>
+          <t>Market Segmentation</t>
+        </is>
+      </c>
+      <c r="F70" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr"/>
+      <c r="H70" s="2" t="inlineStr"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="2" t="inlineStr">
+        <is>
+          <t>Business Studies</t>
+        </is>
+      </c>
+      <c r="B71" s="2" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+      <c r="C71" s="2" t="inlineStr">
+        <is>
+          <t>Business Activity, Marketing &amp; People</t>
+        </is>
+      </c>
+      <c r="D71" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E71" s="12" t="inlineStr">
+        <is>
+          <t>Product &amp; the Product Life Cycle</t>
+        </is>
+      </c>
+      <c r="F71" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G71" s="2" t="inlineStr"/>
+      <c r="H71" s="2" t="inlineStr"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="2" t="inlineStr">
+        <is>
+          <t>Business Studies</t>
+        </is>
+      </c>
+      <c r="B72" s="2" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+      <c r="C72" s="2" t="inlineStr">
+        <is>
+          <t>Business Activity, Marketing &amp; People</t>
+        </is>
+      </c>
+      <c r="D72" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E72" s="12" t="inlineStr">
+        <is>
+          <t>Pricing Methods</t>
+        </is>
+      </c>
+      <c r="F72" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G72" s="2" t="inlineStr"/>
+      <c r="H72" s="2" t="inlineStr"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="2" t="inlineStr">
+        <is>
+          <t>Business Studies</t>
+        </is>
+      </c>
+      <c r="B73" s="2" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+      <c r="C73" s="2" t="inlineStr">
+        <is>
+          <t>Business Activity, Marketing &amp; People</t>
+        </is>
+      </c>
+      <c r="D73" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E73" s="12" t="inlineStr">
+        <is>
+          <t>Promotion &amp; Place</t>
+        </is>
+      </c>
+      <c r="F73" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G73" s="2" t="inlineStr"/>
+      <c r="H73" s="2" t="inlineStr"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="2" t="inlineStr">
+        <is>
+          <t>Business Studies</t>
+        </is>
+      </c>
+      <c r="B74" s="2" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+      <c r="C74" s="2" t="inlineStr">
+        <is>
+          <t>Business Activity, Marketing &amp; People</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E74" s="12" t="inlineStr">
+        <is>
+          <t>The Marketing Mix in Action</t>
+        </is>
+      </c>
+      <c r="F74" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G74" s="2" t="inlineStr"/>
+      <c r="H74" s="2" t="inlineStr"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="2" t="inlineStr">
+        <is>
+          <t>Business Studies</t>
+        </is>
+      </c>
+      <c r="B75" s="2" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+      <c r="C75" s="2" t="inlineStr">
+        <is>
+          <t>Business Activity, Marketing &amp; People</t>
+        </is>
+      </c>
+      <c r="D75" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="E75" s="12" t="inlineStr">
+        <is>
+          <t>Organisational Structures &amp; Ways of Working</t>
+        </is>
+      </c>
+      <c r="F75" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G75" s="2" t="inlineStr"/>
+      <c r="H75" s="2" t="inlineStr"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>Business Studies</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+      <c r="C76" s="2" t="inlineStr">
+        <is>
+          <t>Business Activity, Marketing &amp; People</t>
+        </is>
+      </c>
+      <c r="D76" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="E76" s="12" t="inlineStr">
+        <is>
+          <t>Recruitment, Motivation, Training &amp; Employment Law</t>
+        </is>
+      </c>
+      <c r="F76" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G76" s="2" t="inlineStr"/>
+      <c r="H76" s="2" t="inlineStr"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>Business Studies</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+      <c r="C77" s="2" t="inlineStr">
+        <is>
+          <t>Operations, Finance &amp; Influences on Business</t>
+        </is>
+      </c>
+      <c r="D77" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E77" s="12" t="inlineStr">
+        <is>
+          <t>Production Processes &amp; Technology</t>
+        </is>
+      </c>
+      <c r="F77" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G77" s="2" t="inlineStr"/>
+      <c r="H77" s="2" t="inlineStr"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>Business Studies</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+      <c r="C78" s="2" t="inlineStr">
+        <is>
+          <t>Operations, Finance &amp; Influences on Business</t>
+        </is>
+      </c>
+      <c r="D78" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="E78" s="12" t="inlineStr">
+        <is>
+          <t>Quality of Goods &amp; Services</t>
+        </is>
+      </c>
+      <c r="F78" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G78" s="2" t="inlineStr"/>
+      <c r="H78" s="2" t="inlineStr"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>Business Studies</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+      <c r="C79" s="2" t="inlineStr">
+        <is>
+          <t>Operations, Finance &amp; Influences on Business</t>
+        </is>
+      </c>
+      <c r="D79" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="E79" s="12" t="inlineStr">
+        <is>
+          <t>The Sales Process &amp; Customer Service</t>
+        </is>
+      </c>
+      <c r="F79" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G79" s="2" t="inlineStr"/>
+      <c r="H79" s="2" t="inlineStr"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>Business Studies</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+      <c r="C80" s="2" t="inlineStr">
+        <is>
+          <t>Operations, Finance &amp; Influences on Business</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="E80" s="12" t="inlineStr">
+        <is>
+          <t>Consumer Law</t>
+        </is>
+      </c>
+      <c r="F80" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr"/>
+      <c r="H80" s="2" t="inlineStr"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>Business Studies</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="inlineStr">
+        <is>
+          <t>Operations, Finance &amp; Influences on Business</t>
+        </is>
+      </c>
+      <c r="D81" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E81" s="12" t="inlineStr">
+        <is>
+          <t>Business Location</t>
+        </is>
+      </c>
+      <c r="F81" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G81" s="2" t="inlineStr"/>
+      <c r="H81" s="2" t="inlineStr"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>Business Studies</t>
+        </is>
+      </c>
+      <c r="B82" s="2" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+      <c r="C82" s="2" t="inlineStr">
+        <is>
+          <t>Operations, Finance &amp; Influences on Business</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="E82" s="12" t="inlineStr">
+        <is>
+          <t>Working with Suppliers &amp; Procurement</t>
+        </is>
+      </c>
+      <c r="F82" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr"/>
+      <c r="H82" s="2" t="inlineStr"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="2" t="inlineStr">
+        <is>
+          <t>Business Studies</t>
+        </is>
+      </c>
+      <c r="B83" s="2" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+      <c r="C83" s="2" t="inlineStr">
+        <is>
+          <t>Operations, Finance &amp; Influences on Business</t>
+        </is>
+      </c>
+      <c r="D83" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="E83" s="12" t="inlineStr">
+        <is>
+          <t>The Role of the Finance Function</t>
+        </is>
+      </c>
+      <c r="F83" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G83" s="2" t="inlineStr"/>
+      <c r="H83" s="2" t="inlineStr"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>Business Studies</t>
+        </is>
+      </c>
+      <c r="B84" s="2" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+      <c r="C84" s="2" t="inlineStr">
+        <is>
+          <t>Operations, Finance &amp; Influences on Business</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="E84" s="12" t="inlineStr">
+        <is>
+          <t>Sources of Finance</t>
+        </is>
+      </c>
+      <c r="F84" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr"/>
+      <c r="H84" s="2" t="inlineStr"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
+        <is>
+          <t>Business Studies</t>
+        </is>
+      </c>
+      <c r="B85" s="2" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+      <c r="C85" s="2" t="inlineStr">
+        <is>
+          <t>Operations, Finance &amp; Influences on Business</t>
+        </is>
+      </c>
+      <c r="D85" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="E85" s="12" t="inlineStr">
+        <is>
+          <t>Revenue, Costs &amp; Profit</t>
+        </is>
+      </c>
+      <c r="F85" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G85" s="2" t="inlineStr"/>
+      <c r="H85" s="2" t="inlineStr"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>Business Studies</t>
+        </is>
+      </c>
+      <c r="B86" s="2" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="inlineStr">
+        <is>
+          <t>Operations, Finance &amp; Influences on Business</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="E86" s="12" t="inlineStr">
+        <is>
+          <t>Profit Margins &amp; Average Rate of Return</t>
+        </is>
+      </c>
+      <c r="F86" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr"/>
+      <c r="H86" s="2" t="inlineStr"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
+        <is>
+          <t>Business Studies</t>
+        </is>
+      </c>
+      <c r="B87" s="2" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+      <c r="C87" s="2" t="inlineStr">
+        <is>
+          <t>Operations, Finance &amp; Influences on Business</t>
+        </is>
+      </c>
+      <c r="D87" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="E87" s="12" t="inlineStr">
+        <is>
+          <t>Break-even</t>
+        </is>
+      </c>
+      <c r="F87" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G87" s="2" t="inlineStr"/>
+      <c r="H87" s="2" t="inlineStr"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>Business Studies</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+      <c r="C88" s="2" t="inlineStr">
+        <is>
+          <t>Operations, Finance &amp; Influences on Business</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="E88" s="12" t="inlineStr">
+        <is>
+          <t>Cash &amp; Cash Flow</t>
+        </is>
+      </c>
+      <c r="F88" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr"/>
+      <c r="H88" s="2" t="inlineStr"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>Business Studies</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+      <c r="C89" s="2" t="inlineStr">
+        <is>
+          <t>Operations, Finance &amp; Influences on Business</t>
+        </is>
+      </c>
+      <c r="D89" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="E89" s="12" t="inlineStr">
+        <is>
+          <t>Ethical &amp; Environmental Considerations</t>
+        </is>
+      </c>
+      <c r="F89" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G89" s="2" t="inlineStr"/>
+      <c r="H89" s="2" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>Business Studies</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+      <c r="C90" s="2" t="inlineStr">
+        <is>
+          <t>Operations, Finance &amp; Influences on Business</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="E90" s="12" t="inlineStr">
+        <is>
+          <t>The Economic Climate &amp; Globalisation</t>
+        </is>
+      </c>
+      <c r="F90" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr"/>
+      <c r="H90" s="2" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="inlineStr">
+        <is>
+          <t>Business Studies</t>
+        </is>
+      </c>
+      <c r="B91" s="2" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
+      <c r="C91" s="2" t="inlineStr">
+        <is>
+          <t>Operations, Finance &amp; Influences on Business</t>
+        </is>
+      </c>
+      <c r="D91" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="E91" s="12" t="inlineStr">
+        <is>
+          <t>The Interdependent Nature of Business</t>
+        </is>
+      </c>
+      <c r="F91" s="5" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G91" s="2" t="inlineStr"/>
+      <c r="H91" s="2" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H61"/>
+  <autoFilter ref="A1:H91"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Tracker: register Spanish/French/German AQA as built (free tier)
- _gen_tracker.py NAME_MAP gets the three AQA language entries so the
  spec database matches the new free-tier slugs.
- data/free-tier-status.json appended with the three language entries
  (26 lessons each, Practice format, full hero/practice/related-media
  coverage).
- data/gcse-subject-tracker.xlsx regenerated from current state.

Tracker totals: 193 specs, 29 built (+3 from this migration).

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/gcse-subject-tracker.xlsx
+++ b/data/gcse-subject-tracker.xlsx
@@ -5685,24 +5685,54 @@
           <t>Practice</t>
         </is>
       </c>
-      <c r="F88" s="6" t="inlineStr">
-        <is>
-          <t>Not built</t>
-        </is>
-      </c>
-      <c r="G88" s="2" t="inlineStr"/>
-      <c r="H88" s="6" t="inlineStr">
-        <is>
-          <t>Needs building</t>
-        </is>
-      </c>
-      <c r="I88" s="2" t="inlineStr"/>
-      <c r="J88" s="2" t="inlineStr"/>
-      <c r="K88" s="2" t="inlineStr"/>
-      <c r="L88" s="2" t="inlineStr"/>
-      <c r="M88" s="2" t="inlineStr"/>
-      <c r="N88" s="2" t="inlineStr"/>
-      <c r="O88" s="2" t="inlineStr"/>
+      <c r="F88" s="5" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="H88" s="5" t="inlineStr">
+        <is>
+          <t>26/26</t>
+        </is>
+      </c>
+      <c r="I88" s="5" t="inlineStr">
+        <is>
+          <t>26/26</t>
+        </is>
+      </c>
+      <c r="J88" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K88" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L88" s="5" t="inlineStr">
+        <is>
+          <t>26/26</t>
+        </is>
+      </c>
+      <c r="M88" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N88" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O88" s="2" t="inlineStr">
+        <is>
+          <t>Per-problem flag</t>
+        </is>
+      </c>
       <c r="P88" s="2" t="inlineStr"/>
       <c r="Q88" s="2" t="inlineStr"/>
       <c r="R88" s="2" t="inlineStr"/>
@@ -6341,24 +6371,54 @@
           <t>Practice</t>
         </is>
       </c>
-      <c r="F101" s="6" t="inlineStr">
-        <is>
-          <t>Not built</t>
-        </is>
-      </c>
-      <c r="G101" s="2" t="inlineStr"/>
-      <c r="H101" s="6" t="inlineStr">
-        <is>
-          <t>Needs building</t>
-        </is>
-      </c>
-      <c r="I101" s="2" t="inlineStr"/>
-      <c r="J101" s="2" t="inlineStr"/>
-      <c r="K101" s="2" t="inlineStr"/>
-      <c r="L101" s="2" t="inlineStr"/>
-      <c r="M101" s="2" t="inlineStr"/>
-      <c r="N101" s="2" t="inlineStr"/>
-      <c r="O101" s="2" t="inlineStr"/>
+      <c r="F101" s="5" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="G101" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="H101" s="5" t="inlineStr">
+        <is>
+          <t>26/26</t>
+        </is>
+      </c>
+      <c r="I101" s="5" t="inlineStr">
+        <is>
+          <t>26/26</t>
+        </is>
+      </c>
+      <c r="J101" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K101" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L101" s="5" t="inlineStr">
+        <is>
+          <t>26/26</t>
+        </is>
+      </c>
+      <c r="M101" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N101" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O101" s="2" t="inlineStr">
+        <is>
+          <t>Per-problem flag</t>
+        </is>
+      </c>
       <c r="P101" s="2" t="inlineStr"/>
       <c r="Q101" s="2" t="inlineStr"/>
       <c r="R101" s="2" t="inlineStr"/>
@@ -9157,24 +9217,54 @@
           <t>Practice</t>
         </is>
       </c>
-      <c r="F154" s="6" t="inlineStr">
-        <is>
-          <t>Not built</t>
-        </is>
-      </c>
-      <c r="G154" s="2" t="inlineStr"/>
-      <c r="H154" s="6" t="inlineStr">
-        <is>
-          <t>Needs building</t>
-        </is>
-      </c>
-      <c r="I154" s="2" t="inlineStr"/>
-      <c r="J154" s="2" t="inlineStr"/>
-      <c r="K154" s="2" t="inlineStr"/>
-      <c r="L154" s="2" t="inlineStr"/>
-      <c r="M154" s="2" t="inlineStr"/>
-      <c r="N154" s="2" t="inlineStr"/>
-      <c r="O154" s="2" t="inlineStr"/>
+      <c r="F154" s="5" t="inlineStr">
+        <is>
+          <t>Built</t>
+        </is>
+      </c>
+      <c r="G154" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="H154" s="5" t="inlineStr">
+        <is>
+          <t>26/26</t>
+        </is>
+      </c>
+      <c r="I154" s="5" t="inlineStr">
+        <is>
+          <t>26/26</t>
+        </is>
+      </c>
+      <c r="J154" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="K154" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="L154" s="5" t="inlineStr">
+        <is>
+          <t>26/26</t>
+        </is>
+      </c>
+      <c r="M154" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="N154" s="2" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="O154" s="2" t="inlineStr">
+        <is>
+          <t>Per-problem flag</t>
+        </is>
+      </c>
       <c r="P154" s="2" t="inlineStr"/>
       <c r="Q154" s="2" t="inlineStr"/>
       <c r="R154" s="2" t="inlineStr"/>

</xml_diff>